<commit_message>
major changes in unsupervised and supervised analysis
</commit_message>
<xml_diff>
--- a/data/Vitrificados do PIA - Dados de inspeção.xlsx
+++ b/data/Vitrificados do PIA - Dados de inspeção.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GabrielFalcone\Desktop\dev-folders\bayer-cristalizadores\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72935F97-2B59-4CCE-9F87-445A487FA468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ECF3E65-1E08-4A36-A2D5-8624F8CF3DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{6032B5C1-9728-42CC-9E3A-B210895B9ABF}"/>
   </bookViews>
@@ -18,9 +18,9 @@
     <sheet name="30-351" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'30-151'!$A$4:$I$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'30-251'!$A$4:$I$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'30-351'!$A$4:$I$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'30-151'!$A$4:$J$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'30-251'!$A$4:$J$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'30-351'!$A$4:$J$35</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="308">
   <si>
     <t>ANO</t>
   </si>
@@ -1178,11 +1178,20 @@
   <si>
     <t>08/05 e 12 - 28/05/2020</t>
   </si>
+  <si>
+    <t>DATA ANCORADA NA SÉRIE DE FERRO</t>
+  </si>
+  <si>
+    <t>Fora do Período da Série</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy\ hh:mm:ss"/>
+  </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1834,7 +1843,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2029,13 +2038,47 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2113,6 +2156,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2122,22 +2174,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2501,33 +2562,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95902C09-C2A0-4C8D-B3D6-67337859EB2A}">
-  <dimension ref="A1:U41"/>
+  <dimension ref="A1:V41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.109375" customWidth="1"/>
     <col min="2" max="2" width="16.44140625" customWidth="1"/>
-    <col min="3" max="3" width="32.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="44.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="91.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="48.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="56.44140625" style="76" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.33203125" customWidth="1"/>
+    <col min="5" max="7" width="16.44140625" customWidth="1"/>
+    <col min="8" max="8" width="36.77734375" customWidth="1"/>
+    <col min="9" max="9" width="80.21875" customWidth="1"/>
+    <col min="10" max="10" width="39.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="75" t="s">
+    <row r="1" spans="1:22" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="87" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="77"/>
-      <c r="J1" s="1"/>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="89"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
@@ -2539,18 +2599,19 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
-    </row>
-    <row r="2" spans="1:21" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="78"/>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="80"/>
-      <c r="J2" s="1"/>
+      <c r="V1" s="1"/>
+    </row>
+    <row r="2" spans="1:22" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="90"/>
+      <c r="B2" s="91"/>
+      <c r="C2" s="91"/>
+      <c r="D2" s="91"/>
+      <c r="E2" s="91"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="91"/>
+      <c r="H2" s="91"/>
+      <c r="I2" s="91"/>
+      <c r="J2" s="92"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
@@ -2562,18 +2623,19 @@
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
       <c r="U2" s="1"/>
-    </row>
-    <row r="3" spans="1:21" ht="14.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="81"/>
-      <c r="B3" s="82"/>
-      <c r="C3" s="82"/>
-      <c r="D3" s="82"/>
-      <c r="E3" s="82"/>
-      <c r="F3" s="82"/>
-      <c r="G3" s="82"/>
-      <c r="H3" s="82"/>
-      <c r="I3" s="83"/>
-      <c r="J3" s="1"/>
+      <c r="V2" s="1"/>
+    </row>
+    <row r="3" spans="1:22" ht="14.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="93"/>
+      <c r="B3" s="94"/>
+      <c r="C3" s="94"/>
+      <c r="D3" s="94"/>
+      <c r="E3" s="94"/>
+      <c r="F3" s="94"/>
+      <c r="G3" s="94"/>
+      <c r="H3" s="94"/>
+      <c r="I3" s="94"/>
+      <c r="J3" s="95"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
@@ -2585,250 +2647,278 @@
       <c r="S3" s="1"/>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
-    </row>
-    <row r="4" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="V3" s="1"/>
+    </row>
+    <row r="4" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="66" t="s">
+        <v>306</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="J4" s="8" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A5" s="91">
+    <row r="5" spans="1:22" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="103">
         <v>2004</v>
       </c>
       <c r="B5" s="11">
         <v>38021</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D5" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="D5" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="E5" s="11"/>
+      <c r="E5" s="11" t="s">
+        <v>210</v>
+      </c>
       <c r="F5" s="11"/>
-      <c r="G5" s="12" t="s">
+      <c r="G5" s="11"/>
+      <c r="H5" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="I5" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="I5" s="13" t="s">
+      <c r="J5" s="13" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="92"/>
+    <row r="6" spans="1:22" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="104"/>
       <c r="B6" s="14">
         <v>38069</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="68" t="s">
+        <v>307</v>
+      </c>
+      <c r="D6" s="14" t="s">
         <v>220</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="E6" s="14" t="s">
         <v>211</v>
       </c>
-      <c r="E6" s="14" t="s">
-        <v>210</v>
-      </c>
-      <c r="F6" s="14"/>
-      <c r="G6" s="15" t="s">
+      <c r="F6" s="14" t="s">
+        <v>210</v>
+      </c>
+      <c r="G6" s="14"/>
+      <c r="H6" s="15" t="s">
         <v>200</v>
       </c>
-      <c r="H6" s="15" t="s">
+      <c r="I6" s="15" t="s">
         <v>201</v>
       </c>
-      <c r="I6" s="16" t="s">
+      <c r="J6" s="16" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="87" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="92"/>
+    <row r="7" spans="1:22" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="104"/>
       <c r="B7" s="14">
         <v>38072</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="68" t="s">
+        <v>307</v>
+      </c>
+      <c r="D7" s="14" t="s">
         <v>220</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="E7" s="14" t="s">
         <v>211</v>
       </c>
-      <c r="E7" s="14" t="s">
-        <v>210</v>
-      </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="15" t="s">
+      <c r="F7" s="14" t="s">
+        <v>210</v>
+      </c>
+      <c r="G7" s="14"/>
+      <c r="H7" s="15" t="s">
         <v>202</v>
       </c>
-      <c r="H7" s="15" t="s">
+      <c r="I7" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="I7" s="17" t="s">
+      <c r="J7" s="17" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="93"/>
+    <row r="8" spans="1:22" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="105"/>
       <c r="B8" s="18">
         <v>38281</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="69" t="s">
+        <v>307</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>220</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="E8" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18" t="s">
-        <v>210</v>
-      </c>
-      <c r="G8" s="19" t="s">
+      <c r="F8" s="18"/>
+      <c r="G8" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="H8" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="I8" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="I8" s="20" t="s">
+      <c r="J8" s="20" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="72" x14ac:dyDescent="0.3">
-      <c r="A9" s="84">
+    <row r="9" spans="1:22" ht="72" x14ac:dyDescent="0.3">
+      <c r="A9" s="96">
         <v>2006</v>
       </c>
       <c r="B9" s="11">
         <v>38744</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D9" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="E9" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="E9" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="F9" s="11"/>
-      <c r="G9" s="12" t="s">
+      <c r="F9" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="G9" s="11"/>
+      <c r="H9" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="H9" s="12" t="s">
+      <c r="I9" s="12" t="s">
         <v>244</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="J9" s="13" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="85"/>
+    <row r="10" spans="1:22" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="97"/>
       <c r="B10" s="18">
         <v>38960</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="69" t="s">
+        <v>307</v>
+      </c>
+      <c r="D10" s="18" t="s">
         <v>219</v>
       </c>
-      <c r="D10" s="18" t="s">
-        <v>210</v>
-      </c>
       <c r="E10" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="F10" s="18"/>
-      <c r="G10" s="19" t="s">
+      <c r="F10" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="G10" s="18"/>
+      <c r="H10" s="19" t="s">
         <v>248</v>
       </c>
-      <c r="H10" s="19" t="s">
+      <c r="I10" s="19" t="s">
         <v>246</v>
       </c>
-      <c r="I10" s="17" t="s">
+      <c r="J10" s="17" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="89">
+    <row r="11" spans="1:22" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="101">
         <v>2007</v>
       </c>
       <c r="B11" s="21">
         <v>39294</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="70" t="s">
+        <v>307</v>
+      </c>
+      <c r="D11" s="21" t="s">
         <v>219</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="E11" s="21" t="s">
         <v>211</v>
       </c>
-      <c r="E11" s="21" t="s">
-        <v>210</v>
-      </c>
-      <c r="F11" s="21"/>
-      <c r="G11" s="22" t="s">
+      <c r="F11" s="21" t="s">
+        <v>210</v>
+      </c>
+      <c r="G11" s="21"/>
+      <c r="H11" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="H11" s="22" t="s">
+      <c r="I11" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="I11" s="23" t="s">
+      <c r="J11" s="23" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="90"/>
+    <row r="12" spans="1:22" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="102"/>
       <c r="B12" s="18">
         <v>39325</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="69" t="s">
+        <v>307</v>
+      </c>
+      <c r="D12" s="18" t="s">
         <v>219</v>
       </c>
-      <c r="D12" s="18" t="s">
-        <v>210</v>
-      </c>
       <c r="E12" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="F12" s="18"/>
-      <c r="G12" s="19" t="s">
+      <c r="F12" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="G12" s="18"/>
+      <c r="H12" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="H12" s="19"/>
-      <c r="I12" s="17" t="s">
+      <c r="I12" s="19"/>
+      <c r="J12" s="17" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="72" x14ac:dyDescent="0.3">
-      <c r="A13" s="72">
+    <row r="13" spans="1:22" ht="72" x14ac:dyDescent="0.3">
+      <c r="A13" s="84">
         <v>2008</v>
       </c>
       <c r="B13" s="11">
         <v>39452</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>250</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>211</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>211</v>
@@ -2836,97 +2926,108 @@
       <c r="F13" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="G13" s="12" t="s">
+      <c r="G13" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="H13" s="12" t="s">
         <v>213</v>
       </c>
-      <c r="H13" s="12" t="s">
+      <c r="I13" s="12" t="s">
         <v>214</v>
       </c>
-      <c r="I13" s="13" t="s">
+      <c r="J13" s="13" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="74"/>
-      <c r="B14" s="66">
+    <row r="14" spans="1:22" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="86"/>
+      <c r="B14" s="106">
         <v>39491</v>
       </c>
-      <c r="C14" s="66" t="s">
+      <c r="C14" s="112" t="s">
+        <v>307</v>
+      </c>
+      <c r="D14" s="106" t="s">
         <v>219</v>
       </c>
-      <c r="D14" s="66" t="s">
+      <c r="E14" s="106" t="s">
         <v>211</v>
       </c>
-      <c r="E14" s="66" t="s">
-        <v>210</v>
-      </c>
-      <c r="F14" s="66"/>
-      <c r="G14" s="69" t="s">
+      <c r="F14" s="106" t="s">
+        <v>210</v>
+      </c>
+      <c r="G14" s="106"/>
+      <c r="H14" s="81" t="s">
         <v>252</v>
       </c>
-      <c r="H14" s="69" t="s">
+      <c r="I14" s="81" t="s">
         <v>253</v>
       </c>
-      <c r="I14" s="94" t="s">
+      <c r="J14" s="109" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="74"/>
-      <c r="B15" s="67"/>
-      <c r="C15" s="67"/>
-      <c r="D15" s="67"/>
-      <c r="E15" s="67"/>
-      <c r="F15" s="67"/>
-      <c r="G15" s="70"/>
-      <c r="H15" s="70"/>
-      <c r="I15" s="95"/>
-    </row>
-    <row r="16" spans="1:21" ht="284.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="74"/>
-      <c r="B16" s="68"/>
-      <c r="C16" s="68"/>
-      <c r="D16" s="68"/>
-      <c r="E16" s="68"/>
-      <c r="F16" s="68"/>
-      <c r="G16" s="71"/>
-      <c r="H16" s="71"/>
-      <c r="I16" s="96"/>
-    </row>
-    <row r="17" spans="1:9" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="73"/>
+    <row r="15" spans="1:22" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="86"/>
+      <c r="B15" s="107"/>
+      <c r="C15" s="113"/>
+      <c r="D15" s="107"/>
+      <c r="E15" s="107"/>
+      <c r="F15" s="107"/>
+      <c r="G15" s="107"/>
+      <c r="H15" s="82"/>
+      <c r="I15" s="82"/>
+      <c r="J15" s="110"/>
+    </row>
+    <row r="16" spans="1:22" ht="284.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="86"/>
+      <c r="B16" s="108"/>
+      <c r="C16" s="114"/>
+      <c r="D16" s="108"/>
+      <c r="E16" s="108"/>
+      <c r="F16" s="108"/>
+      <c r="G16" s="108"/>
+      <c r="H16" s="83"/>
+      <c r="I16" s="83"/>
+      <c r="J16" s="111"/>
+    </row>
+    <row r="17" spans="1:10" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="85"/>
       <c r="B17" s="18">
         <v>39602</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="69" t="s">
+        <v>307</v>
+      </c>
+      <c r="D17" s="18" t="s">
         <v>219</v>
       </c>
-      <c r="D17" s="18" t="s">
-        <v>210</v>
-      </c>
-      <c r="E17" s="18"/>
+      <c r="E17" s="18" t="s">
+        <v>210</v>
+      </c>
       <c r="F17" s="18"/>
-      <c r="G17" s="19" t="s">
+      <c r="G17" s="18"/>
+      <c r="H17" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="H17" s="19"/>
-      <c r="I17" s="17" t="s">
+      <c r="I17" s="19"/>
+      <c r="J17" s="17" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="273.60000000000002" x14ac:dyDescent="0.3">
-      <c r="A18" s="86">
+    <row r="18" spans="1:10" ht="273.60000000000002" x14ac:dyDescent="0.3">
+      <c r="A18" s="98">
         <v>2009</v>
       </c>
       <c r="B18" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D18" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="D18" s="12" t="s">
-        <v>210</v>
-      </c>
       <c r="E18" s="12" t="s">
         <v>210</v>
       </c>
@@ -2934,580 +3035,657 @@
         <v>210</v>
       </c>
       <c r="G18" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="H18" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="H18" s="12" t="s">
+      <c r="I18" s="12" t="s">
         <v>254</v>
       </c>
-      <c r="I18" s="13" t="s">
+      <c r="J18" s="13" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="87"/>
+    <row r="19" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="99"/>
       <c r="B19" s="14">
         <v>39909</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="68" t="s">
+        <v>307</v>
+      </c>
+      <c r="D19" s="14" t="s">
         <v>221</v>
       </c>
-      <c r="D19" s="14" t="s">
-        <v>210</v>
-      </c>
-      <c r="E19" s="14"/>
+      <c r="E19" s="14" t="s">
+        <v>210</v>
+      </c>
       <c r="F19" s="14"/>
-      <c r="G19" s="15" t="s">
+      <c r="G19" s="14"/>
+      <c r="H19" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="H19" s="15" t="s">
+      <c r="I19" s="15" t="s">
         <v>256</v>
       </c>
-      <c r="I19" s="16" t="s">
+      <c r="J19" s="16" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="259.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="88"/>
+    <row r="20" spans="1:10" ht="259.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="100"/>
       <c r="B20" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C20" s="19" t="s">
+      <c r="C20" s="69" t="s">
+        <v>307</v>
+      </c>
+      <c r="D20" s="19" t="s">
         <v>219</v>
       </c>
-      <c r="D20" s="19" t="s">
+      <c r="E20" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="E20" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19" t="s">
+      <c r="F20" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19" t="s">
         <v>222</v>
       </c>
-      <c r="H20" s="19" t="s">
+      <c r="I20" s="19" t="s">
         <v>257</v>
       </c>
-      <c r="I20" s="17" t="s">
+      <c r="J20" s="17" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="30">
         <v>2010</v>
       </c>
       <c r="B21" s="11">
         <v>40372</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D21" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="E21" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="G21" s="12"/>
-      <c r="H21" s="12" t="s">
+      <c r="F21" s="11"/>
+      <c r="G21" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="I21" s="13" t="s">
+      <c r="J21" s="13" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="10">
         <v>2011</v>
       </c>
       <c r="B22" s="26" t="s">
         <v>225</v>
       </c>
-      <c r="C22" s="26" t="s">
+      <c r="C22" s="72">
+        <v>40692.482199074075</v>
+      </c>
+      <c r="D22" s="26" t="s">
         <v>219</v>
       </c>
-      <c r="D22" s="26" t="s">
-        <v>210</v>
-      </c>
-      <c r="E22" s="26"/>
+      <c r="E22" s="26" t="s">
+        <v>210</v>
+      </c>
       <c r="F22" s="26"/>
-      <c r="G22" s="26" t="s">
+      <c r="G22" s="26"/>
+      <c r="H22" s="26" t="s">
         <v>224</v>
       </c>
-      <c r="H22" s="26" t="s">
+      <c r="I22" s="26" t="s">
         <v>150</v>
       </c>
-      <c r="I22" s="27" t="s">
+      <c r="J22" s="27" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="48">
         <v>2012</v>
       </c>
       <c r="B23" s="49">
         <v>41064</v>
       </c>
-      <c r="C23" s="35" t="s">
+      <c r="C23" s="73">
+        <v>41071.448611111111</v>
+      </c>
+      <c r="D23" s="35" t="s">
         <v>220</v>
       </c>
-      <c r="D23" s="35" t="s">
+      <c r="E23" s="35" t="s">
         <v>211</v>
       </c>
-      <c r="E23" s="35"/>
       <c r="F23" s="35"/>
-      <c r="G23" s="26" t="s">
+      <c r="G23" s="35"/>
+      <c r="H23" s="26" t="s">
         <v>151</v>
       </c>
-      <c r="H23" s="26"/>
-      <c r="I23" s="27"/>
-    </row>
-    <row r="24" spans="1:9" ht="216" x14ac:dyDescent="0.3">
-      <c r="A24" s="86">
+      <c r="I23" s="26"/>
+      <c r="J23" s="27"/>
+    </row>
+    <row r="24" spans="1:10" ht="216" x14ac:dyDescent="0.3">
+      <c r="A24" s="98">
         <v>2013</v>
       </c>
       <c r="B24" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="C24" s="12" t="s">
+      <c r="C24" s="67">
+        <v>41358</v>
+      </c>
+      <c r="D24" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="D24" s="12" t="s">
+      <c r="E24" s="12" t="s">
         <v>211</v>
       </c>
-      <c r="E24" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="F24" s="12"/>
-      <c r="G24" s="12" t="s">
+      <c r="F24" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="H24" s="32" t="s">
+      <c r="I24" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="I24" s="13" t="s">
+      <c r="J24" s="13" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="87"/>
+    <row r="25" spans="1:10" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A25" s="99"/>
       <c r="B25" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="C25" s="15" t="s">
+      <c r="C25" s="68">
+        <v>41451.179861111108</v>
+      </c>
+      <c r="D25" s="15" t="s">
         <v>219</v>
       </c>
-      <c r="D25" s="15" t="s">
-        <v>210</v>
-      </c>
-      <c r="E25" s="15"/>
+      <c r="E25" s="15" t="s">
+        <v>210</v>
+      </c>
       <c r="F25" s="15"/>
-      <c r="G25" s="15" t="s">
+      <c r="G25" s="15"/>
+      <c r="H25" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="H25" s="15" t="s">
+      <c r="I25" s="15" t="s">
         <v>227</v>
       </c>
-      <c r="I25" s="16" t="s">
+      <c r="J25" s="16" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="87"/>
+    <row r="26" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A26" s="99"/>
       <c r="B26" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="C26" s="15" t="s">
+      <c r="C26" s="68">
+        <v>41451.179861111108</v>
+      </c>
+      <c r="D26" s="15" t="s">
         <v>229</v>
       </c>
-      <c r="D26" s="15" t="s">
+      <c r="E26" s="15" t="s">
         <v>211</v>
       </c>
-      <c r="E26" s="15"/>
       <c r="F26" s="15"/>
-      <c r="G26" s="15" t="s">
+      <c r="G26" s="15"/>
+      <c r="H26" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="H26" s="15" t="s">
+      <c r="I26" s="15" t="s">
         <v>231</v>
       </c>
-      <c r="I26" s="16" t="s">
+      <c r="J26" s="16" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="159" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="88"/>
+    <row r="27" spans="1:10" ht="159" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="100"/>
       <c r="B27" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="C27" s="19" t="s">
+      <c r="C27" s="68">
+        <v>41451.179861111108</v>
+      </c>
+      <c r="D27" s="19" t="s">
         <v>233</v>
       </c>
-      <c r="D27" s="19" t="s">
+      <c r="E27" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="E27" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19" t="s">
+      <c r="F27" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="G27" s="19"/>
+      <c r="H27" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="H27" s="19"/>
-      <c r="I27" s="17" t="s">
+      <c r="I27" s="19"/>
+      <c r="J27" s="17" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A28" s="72">
+    <row r="28" spans="1:10" ht="231" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="84">
         <v>2015</v>
       </c>
       <c r="B28" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="C28" s="12" t="s">
+      <c r="C28" s="67">
+        <v>42128.171527777777</v>
+      </c>
+      <c r="D28" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="D28" s="12" t="s">
+      <c r="E28" s="12" t="s">
         <v>211</v>
       </c>
-      <c r="E28" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="F28" s="12"/>
-      <c r="G28" s="12" t="s">
+      <c r="F28" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="H28" s="12" t="s">
+      <c r="I28" s="12" t="s">
         <v>236</v>
       </c>
-      <c r="I28" s="13" t="s">
+      <c r="J28" s="13" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="73"/>
+    <row r="29" spans="1:10" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="85"/>
       <c r="B29" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="C29" s="19" t="s">
+      <c r="C29" s="67">
+        <v>42128.171527777777</v>
+      </c>
+      <c r="D29" s="19" t="s">
         <v>219</v>
       </c>
-      <c r="D29" s="19" t="s">
+      <c r="E29" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="E29" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="F29" s="19"/>
-      <c r="G29" s="19" t="s">
+      <c r="F29" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="G29" s="19"/>
+      <c r="H29" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="H29" s="19" t="s">
+      <c r="I29" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="I29" s="17" t="s">
+      <c r="J29" s="17" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="187.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" ht="187.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="10">
         <v>2016</v>
       </c>
       <c r="B30" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="C30" s="26" t="s">
+      <c r="C30" s="72">
+        <v>42526.429166666669</v>
+      </c>
+      <c r="D30" s="26" t="s">
         <v>219</v>
       </c>
-      <c r="D30" s="26" t="s">
+      <c r="E30" s="26" t="s">
         <v>211</v>
       </c>
-      <c r="E30" s="26" t="s">
-        <v>210</v>
-      </c>
-      <c r="F30" s="26"/>
+      <c r="F30" s="26" t="s">
+        <v>210</v>
+      </c>
       <c r="G30" s="26"/>
-      <c r="H30" s="26" t="s">
+      <c r="H30" s="26"/>
+      <c r="I30" s="26" t="s">
         <v>239</v>
       </c>
-      <c r="I30" s="27" t="s">
+      <c r="J30" s="27" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A31" s="72">
+    <row r="31" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="84">
         <v>2017</v>
       </c>
       <c r="B31" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="C31" s="12" t="s">
+      <c r="C31" s="67">
+        <v>42788.769444444442</v>
+      </c>
+      <c r="D31" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="D31" s="12" t="s">
-        <v>210</v>
-      </c>
       <c r="E31" s="12" t="s">
         <v>210</v>
       </c>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12" t="s">
+      <c r="F31" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="G31" s="12"/>
+      <c r="H31" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="H31" s="12" t="s">
+      <c r="I31" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="I31" s="13" t="s">
+      <c r="J31" s="13" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="74"/>
+    <row r="32" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A32" s="86"/>
       <c r="B32" s="14">
         <v>42818</v>
       </c>
-      <c r="C32" s="14" t="s">
+      <c r="C32" s="68">
+        <v>42817.134027777778</v>
+      </c>
+      <c r="D32" s="14" t="s">
         <v>219</v>
       </c>
-      <c r="D32" s="14" t="s">
+      <c r="E32" s="14" t="s">
         <v>211</v>
       </c>
-      <c r="E32" s="14"/>
       <c r="F32" s="14"/>
-      <c r="G32" s="15" t="s">
+      <c r="G32" s="14"/>
+      <c r="H32" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="H32" s="15" t="s">
+      <c r="I32" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="I32" s="16"/>
-    </row>
-    <row r="33" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A33" s="74"/>
+      <c r="J32" s="16"/>
+    </row>
+    <row r="33" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A33" s="86"/>
       <c r="B33" s="14">
         <v>42937</v>
       </c>
-      <c r="C33" s="14" t="s">
+      <c r="C33" s="68">
+        <v>42933.776388888888</v>
+      </c>
+      <c r="D33" s="14" t="s">
         <v>219</v>
       </c>
-      <c r="D33" s="14" t="s">
-        <v>210</v>
-      </c>
-      <c r="E33" s="14"/>
+      <c r="E33" s="14" t="s">
+        <v>210</v>
+      </c>
       <c r="F33" s="14"/>
-      <c r="G33" s="15"/>
-      <c r="H33" s="15" t="s">
+      <c r="G33" s="14"/>
+      <c r="H33" s="15"/>
+      <c r="I33" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="I33" s="16" t="s">
+      <c r="J33" s="16" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="73"/>
+    <row r="34" spans="1:10" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="85"/>
       <c r="B34" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="C34" s="19" t="s">
+      <c r="C34" s="68">
+        <v>42933.776388888888</v>
+      </c>
+      <c r="D34" s="19" t="s">
         <v>219</v>
       </c>
-      <c r="D34" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="E34" s="19"/>
+      <c r="E34" s="19" t="s">
+        <v>210</v>
+      </c>
       <c r="F34" s="19"/>
-      <c r="G34" s="19" t="s">
+      <c r="G34" s="19"/>
+      <c r="H34" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="H34" s="19" t="s">
+      <c r="I34" s="19" t="s">
         <v>153</v>
       </c>
-      <c r="I34" s="17"/>
-    </row>
-    <row r="35" spans="1:9" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="J34" s="17"/>
+    </row>
+    <row r="35" spans="1:10" ht="72.599999999999994" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10">
         <v>2018</v>
       </c>
       <c r="B35" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="C35" s="26" t="s">
+      <c r="C35" s="72">
+        <v>43304.031944444447</v>
+      </c>
+      <c r="D35" s="26" t="s">
         <v>219</v>
       </c>
-      <c r="D35" s="26" t="s">
+      <c r="E35" s="26" t="s">
         <v>211</v>
       </c>
-      <c r="E35" s="26" t="s">
-        <v>210</v>
-      </c>
-      <c r="F35" s="26"/>
-      <c r="G35" s="26" t="s">
+      <c r="F35" s="26" t="s">
+        <v>210</v>
+      </c>
+      <c r="G35" s="26"/>
+      <c r="H35" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="H35" s="26" t="s">
+      <c r="I35" s="26" t="s">
         <v>259</v>
       </c>
-      <c r="I35" s="34" t="s">
+      <c r="J35" s="34" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="30">
         <v>2019</v>
       </c>
       <c r="B36" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="C36" s="12" t="s">
+      <c r="C36" s="67">
+        <v>43675.118750000001</v>
+      </c>
+      <c r="D36" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="D36" s="12" t="s">
+      <c r="E36" s="12" t="s">
         <v>211</v>
       </c>
-      <c r="E36" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="F36" s="12"/>
+      <c r="F36" s="12" t="s">
+        <v>210</v>
+      </c>
       <c r="G36" s="12"/>
-      <c r="H36" s="12" t="s">
+      <c r="H36" s="12"/>
+      <c r="I36" s="12" t="s">
         <v>261</v>
       </c>
-      <c r="I36" s="13" t="s">
+      <c r="J36" s="13" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="187.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" ht="187.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="10">
         <v>2020</v>
       </c>
       <c r="B37" s="26" t="s">
         <v>138</v>
       </c>
-      <c r="C37" s="26" t="s">
+      <c r="C37" s="72">
+        <v>43927.521527777775</v>
+      </c>
+      <c r="D37" s="26" t="s">
         <v>219</v>
       </c>
-      <c r="D37" s="26" t="s">
+      <c r="E37" s="26" t="s">
         <v>211</v>
       </c>
-      <c r="E37" s="26" t="s">
-        <v>210</v>
-      </c>
-      <c r="F37" s="26"/>
-      <c r="G37" s="26" t="s">
+      <c r="F37" s="26" t="s">
+        <v>210</v>
+      </c>
+      <c r="G37" s="26"/>
+      <c r="H37" s="26" t="s">
         <v>154</v>
       </c>
-      <c r="H37" s="26" t="s">
+      <c r="I37" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="I37" s="27" t="s">
+      <c r="J37" s="27" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="31">
         <v>2021</v>
       </c>
       <c r="B38" s="35">
         <v>44359</v>
       </c>
-      <c r="C38" s="35" t="s">
+      <c r="C38" s="72">
+        <v>44346.968055555553</v>
+      </c>
+      <c r="D38" s="35" t="s">
         <v>241</v>
       </c>
-      <c r="D38" s="35" t="s">
+      <c r="E38" s="35" t="s">
         <v>211</v>
       </c>
-      <c r="E38" s="35" t="s">
-        <v>210</v>
-      </c>
-      <c r="F38" s="35"/>
-      <c r="G38" s="26" t="s">
+      <c r="F38" s="35" t="s">
+        <v>210</v>
+      </c>
+      <c r="G38" s="35"/>
+      <c r="H38" s="26" t="s">
         <v>263</v>
       </c>
-      <c r="H38" s="26" t="s">
+      <c r="I38" s="26" t="s">
         <v>140</v>
       </c>
-      <c r="I38" s="27" t="s">
+      <c r="J38" s="27" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="10">
         <v>2023</v>
       </c>
       <c r="B39" s="35">
         <v>44960</v>
       </c>
-      <c r="C39" s="35" t="s">
+      <c r="C39" s="72">
+        <v>44955.73333333333</v>
+      </c>
+      <c r="D39" s="35" t="s">
         <v>241</v>
       </c>
-      <c r="D39" s="35" t="s">
-        <v>210</v>
-      </c>
-      <c r="E39" s="35"/>
+      <c r="E39" s="35" t="s">
+        <v>210</v>
+      </c>
       <c r="F39" s="35"/>
-      <c r="G39" s="26" t="s">
+      <c r="G39" s="35"/>
+      <c r="H39" s="26" t="s">
         <v>141</v>
       </c>
-      <c r="H39" s="26"/>
-      <c r="I39" s="26" t="s">
+      <c r="I39" s="26"/>
+      <c r="J39" s="26" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" ht="46.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="31">
         <v>2024</v>
       </c>
       <c r="B40" s="47">
         <v>45324</v>
       </c>
-      <c r="C40" s="47" t="s">
+      <c r="C40" s="74">
+        <v>45311.038888888892</v>
+      </c>
+      <c r="D40" s="47" t="s">
         <v>241</v>
       </c>
-      <c r="D40" s="47" t="s">
+      <c r="E40" s="47" t="s">
         <v>211</v>
       </c>
-      <c r="E40" s="47"/>
-      <c r="F40" s="47" t="s">
-        <v>210</v>
-      </c>
-      <c r="G40" s="26"/>
-      <c r="H40" s="26" t="s">
+      <c r="F40" s="47"/>
+      <c r="G40" s="47" t="s">
+        <v>210</v>
+      </c>
+      <c r="H40" s="26"/>
+      <c r="I40" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="I40" s="27" t="s">
+      <c r="J40" s="27" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="25">
         <v>2025</v>
       </c>
       <c r="B41" s="42">
         <v>46006</v>
       </c>
-      <c r="C41" s="42" t="s">
+      <c r="C41" s="75">
+        <v>45999.056250000001</v>
+      </c>
+      <c r="D41" s="42" t="s">
         <v>241</v>
       </c>
-      <c r="D41" s="42" t="s">
-        <v>210</v>
-      </c>
-      <c r="E41" s="42"/>
+      <c r="E41" s="42" t="s">
+        <v>210</v>
+      </c>
       <c r="F41" s="42"/>
-      <c r="G41" s="43" t="s">
+      <c r="G41" s="42"/>
+      <c r="H41" s="43" t="s">
         <v>145</v>
       </c>
-      <c r="H41" s="43" t="s">
+      <c r="I41" s="43" t="s">
         <v>265</v>
       </c>
-      <c r="I41" s="20" t="s">
+      <c r="J41" s="20" t="s">
         <v>264</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I41" xr:uid="{95902C09-C2A0-4C8D-B3D6-67337859EB2A}"/>
-  <mergeCells count="17">
-    <mergeCell ref="A1:I3"/>
+  <autoFilter ref="A4:J41" xr:uid="{95902C09-C2A0-4C8D-B3D6-67337859EB2A}"/>
+  <mergeCells count="18">
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="H14:H16"/>
+    <mergeCell ref="I14:I16"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A31:A34"/>
+    <mergeCell ref="A1:J3"/>
     <mergeCell ref="A9:A10"/>
     <mergeCell ref="A24:A27"/>
     <mergeCell ref="A18:A20"/>
@@ -3515,15 +3693,11 @@
     <mergeCell ref="A13:A17"/>
     <mergeCell ref="A5:A8"/>
     <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
     <mergeCell ref="D14:D16"/>
-    <mergeCell ref="I14:I16"/>
     <mergeCell ref="E14:E16"/>
+    <mergeCell ref="J14:J16"/>
     <mergeCell ref="F14:F16"/>
     <mergeCell ref="G14:G16"/>
-    <mergeCell ref="H14:H16"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A31:A34"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <headerFooter>
@@ -3534,914 +3708,1024 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1F67599-3BD8-474A-B2DB-71494680CF1C}">
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" customWidth="1"/>
-    <col min="2" max="2" width="14.21875" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="42.6640625" customWidth="1"/>
-    <col min="8" max="8" width="54.21875" customWidth="1"/>
-    <col min="9" max="9" width="43" customWidth="1"/>
-    <col min="10" max="10" width="36.21875" customWidth="1"/>
+    <col min="1" max="1" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="56.44140625" style="76" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="49.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="103.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="73.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="36.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="75" t="s">
+    <row r="1" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="87" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="77"/>
-    </row>
-    <row r="2" spans="1:9" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="78"/>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="80"/>
-    </row>
-    <row r="3" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="81"/>
-      <c r="B3" s="82"/>
-      <c r="C3" s="82"/>
-      <c r="D3" s="82"/>
-      <c r="E3" s="82"/>
-      <c r="F3" s="82"/>
-      <c r="G3" s="82"/>
-      <c r="H3" s="82"/>
-      <c r="I3" s="83"/>
-    </row>
-    <row r="4" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="89"/>
+    </row>
+    <row r="2" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="90"/>
+      <c r="B2" s="91"/>
+      <c r="C2" s="91"/>
+      <c r="D2" s="91"/>
+      <c r="E2" s="91"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="91"/>
+      <c r="H2" s="91"/>
+      <c r="I2" s="91"/>
+      <c r="J2" s="92"/>
+    </row>
+    <row r="3" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="93"/>
+      <c r="B3" s="94"/>
+      <c r="C3" s="94"/>
+      <c r="D3" s="94"/>
+      <c r="E3" s="94"/>
+      <c r="F3" s="94"/>
+      <c r="G3" s="94"/>
+      <c r="H3" s="94"/>
+      <c r="I3" s="94"/>
+      <c r="J3" s="95"/>
+    </row>
+    <row r="4" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="66" t="s">
+        <v>306</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="H4" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="I4" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="J4" s="9" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="130.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="86">
+    <row r="5" spans="1:10" ht="130.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="98">
         <v>2004</v>
       </c>
       <c r="B5" s="11">
         <v>38064</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11" t="s">
+      <c r="C5" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="G5" s="12" t="s">
+      <c r="F5" s="11"/>
+      <c r="G5" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="H5" s="12" t="s">
         <v>206</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="I5" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="I5" s="13"/>
-    </row>
-    <row r="6" spans="1:9" ht="182.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="87"/>
+      <c r="J5" s="13"/>
+    </row>
+    <row r="6" spans="1:10" ht="182.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="99"/>
       <c r="B6" s="14">
         <v>38182</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="68" t="s">
+        <v>307</v>
+      </c>
+      <c r="D6" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>210</v>
-      </c>
-      <c r="E6" s="14"/>
+      <c r="E6" s="14" t="s">
+        <v>210</v>
+      </c>
       <c r="F6" s="14"/>
-      <c r="G6" s="15" t="s">
+      <c r="G6" s="14"/>
+      <c r="H6" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="H6" s="15" t="s">
+      <c r="I6" s="15" t="s">
         <v>280</v>
       </c>
-      <c r="I6" s="16" t="s">
+      <c r="J6" s="16" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="144" x14ac:dyDescent="0.3">
-      <c r="A7" s="87"/>
+    <row r="7" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="99"/>
       <c r="B7" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="68" t="s">
+        <v>307</v>
+      </c>
+      <c r="D7" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>210</v>
-      </c>
-      <c r="E7" s="15"/>
+      <c r="E7" s="15" t="s">
+        <v>210</v>
+      </c>
       <c r="F7" s="15"/>
-      <c r="G7" s="15" t="s">
+      <c r="G7" s="15"/>
+      <c r="H7" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="H7" s="33" t="s">
+      <c r="I7" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="I7" s="16" t="s">
+      <c r="J7" s="16" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="88"/>
+    <row r="8" spans="1:10" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="100"/>
       <c r="B8" s="18">
         <v>38204</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="69" t="s">
+        <v>307</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>279</v>
       </c>
-      <c r="D8" s="18" t="s">
-        <v>210</v>
-      </c>
-      <c r="E8" s="18"/>
+      <c r="E8" s="18" t="s">
+        <v>210</v>
+      </c>
       <c r="F8" s="18"/>
-      <c r="G8" s="50" t="s">
+      <c r="G8" s="18"/>
+      <c r="H8" s="50" t="s">
         <v>157</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="I8" s="19" t="s">
         <v>282</v>
       </c>
-      <c r="I8" s="17" t="s">
+      <c r="J8" s="17" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="159" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="31">
         <v>2005</v>
       </c>
       <c r="B9" s="35">
         <v>38398</v>
       </c>
-      <c r="C9" s="35" t="s">
+      <c r="C9" s="72" t="s">
+        <v>307</v>
+      </c>
+      <c r="D9" s="35" t="s">
         <v>279</v>
       </c>
-      <c r="D9" s="35" t="s">
+      <c r="E9" s="35" t="s">
         <v>211</v>
       </c>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35" t="s">
-        <v>210</v>
-      </c>
-      <c r="G9" s="26" t="s">
+      <c r="F9" s="35"/>
+      <c r="G9" s="35" t="s">
+        <v>210</v>
+      </c>
+      <c r="H9" s="26" t="s">
         <v>159</v>
       </c>
-      <c r="H9" s="26"/>
-      <c r="I9" s="27" t="s">
+      <c r="I9" s="26"/>
+      <c r="J9" s="27" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="10">
         <v>2006</v>
       </c>
       <c r="B10" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" s="72" t="s">
+        <v>307</v>
+      </c>
+      <c r="D10" s="26" t="s">
         <v>283</v>
       </c>
-      <c r="D10" s="26" t="s">
+      <c r="E10" s="26" t="s">
         <v>211</v>
       </c>
-      <c r="E10" s="26"/>
       <c r="F10" s="26"/>
-      <c r="G10" s="26" t="s">
+      <c r="G10" s="26"/>
+      <c r="H10" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="H10" s="26" t="s">
+      <c r="I10" s="26" t="s">
         <v>273</v>
       </c>
-      <c r="I10" s="27"/>
-    </row>
-    <row r="11" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="72">
+      <c r="J10" s="27"/>
+    </row>
+    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="84">
         <v>2007</v>
       </c>
       <c r="B11" s="11">
         <v>39104</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D11" s="11" t="s">
         <v>283</v>
       </c>
-      <c r="D11" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="E11" s="11"/>
+      <c r="E11" s="11" t="s">
+        <v>210</v>
+      </c>
       <c r="F11" s="11"/>
-      <c r="G11" s="12" t="s">
+      <c r="G11" s="11"/>
+      <c r="H11" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="H11" s="12"/>
-      <c r="I11" s="13" t="s">
+      <c r="I11" s="12"/>
+      <c r="J11" s="13" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="74"/>
+    <row r="12" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="86"/>
       <c r="B12" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="68" t="s">
+        <v>307</v>
+      </c>
+      <c r="D12" s="15" t="s">
         <v>283</v>
       </c>
-      <c r="D12" s="15" t="s">
-        <v>210</v>
-      </c>
-      <c r="E12" s="15"/>
+      <c r="E12" s="15" t="s">
+        <v>210</v>
+      </c>
       <c r="F12" s="15"/>
-      <c r="G12" s="15" t="s">
+      <c r="G12" s="15"/>
+      <c r="H12" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="H12" s="15" t="s">
+      <c r="I12" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="I12" s="16" t="s">
+      <c r="J12" s="16" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="73"/>
+    <row r="13" spans="1:10" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="85"/>
       <c r="B13" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="69" t="s">
+        <v>307</v>
+      </c>
+      <c r="D13" s="19" t="s">
         <v>283</v>
       </c>
-      <c r="D13" s="19" t="s">
-        <v>210</v>
-      </c>
       <c r="E13" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19" t="s">
+      <c r="F13" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19" t="s">
         <v>275</v>
       </c>
-      <c r="H13" s="19" t="s">
+      <c r="I13" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="I13" s="17" t="s">
+      <c r="J13" s="17" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="200.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="86">
+    <row r="14" spans="1:10" ht="200.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="98">
         <v>2008</v>
       </c>
-      <c r="B14" s="99" t="s">
+      <c r="B14" s="115" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="99" t="s">
+      <c r="C14" s="77" t="s">
+        <v>307</v>
+      </c>
+      <c r="D14" s="115" t="s">
         <v>279</v>
       </c>
-      <c r="D14" s="99" t="s">
+      <c r="E14" s="115" t="s">
         <v>211</v>
       </c>
-      <c r="E14" s="99" t="s">
-        <v>210</v>
-      </c>
-      <c r="F14" s="99"/>
-      <c r="G14" s="99" t="s">
+      <c r="F14" s="115" t="s">
+        <v>210</v>
+      </c>
+      <c r="G14" s="115"/>
+      <c r="H14" s="115" t="s">
         <v>284</v>
       </c>
-      <c r="H14" s="99" t="s">
+      <c r="I14" s="115" t="s">
         <v>54</v>
       </c>
-      <c r="I14" s="101" t="s">
+      <c r="J14" s="117" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="56.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="87"/>
-      <c r="B15" s="100"/>
-      <c r="C15" s="100"/>
-      <c r="D15" s="100"/>
-      <c r="E15" s="100"/>
-      <c r="F15" s="100"/>
-      <c r="G15" s="100"/>
-      <c r="H15" s="100"/>
-      <c r="I15" s="102"/>
-    </row>
-    <row r="16" spans="1:9" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" ht="56.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="99"/>
+      <c r="B15" s="116"/>
+      <c r="C15" s="75" t="s">
+        <v>307</v>
+      </c>
+      <c r="D15" s="116"/>
+      <c r="E15" s="116"/>
+      <c r="F15" s="116"/>
+      <c r="G15" s="116"/>
+      <c r="H15" s="116"/>
+      <c r="I15" s="116"/>
+      <c r="J15" s="118"/>
+    </row>
+    <row r="16" spans="1:10" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="30">
         <v>2009</v>
       </c>
       <c r="B16" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D16" s="12" t="s">
         <v>283</v>
       </c>
-      <c r="D16" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="E16" s="12"/>
+      <c r="E16" s="12" t="s">
+        <v>210</v>
+      </c>
       <c r="F16" s="12"/>
-      <c r="G16" s="12" t="s">
+      <c r="G16" s="12"/>
+      <c r="H16" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="H16" s="12" t="s">
+      <c r="I16" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="I16" s="13" t="s">
+      <c r="J16" s="13" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="86">
+    <row r="17" spans="1:10" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="98">
         <v>2011</v>
       </c>
       <c r="B17" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="C17" s="45" t="s">
+      <c r="C17" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D17" s="45" t="s">
         <v>283</v>
       </c>
-      <c r="D17" s="45" t="s">
-        <v>210</v>
-      </c>
-      <c r="E17" s="45"/>
+      <c r="E17" s="45" t="s">
+        <v>210</v>
+      </c>
       <c r="F17" s="45"/>
-      <c r="G17" s="45" t="s">
+      <c r="G17" s="45"/>
+      <c r="H17" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="H17" s="45" t="s">
+      <c r="I17" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="I17" s="46" t="s">
+      <c r="J17" s="46" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A18" s="87"/>
+    <row r="18" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="99"/>
       <c r="B18" s="14">
         <v>40763</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="68">
+        <v>40762.775694444441</v>
+      </c>
+      <c r="D18" s="14" t="s">
         <v>283</v>
       </c>
-      <c r="D18" s="24" t="s">
-        <v>210</v>
-      </c>
       <c r="E18" s="24" t="s">
         <v>210</v>
       </c>
-      <c r="F18" s="14" t="s">
-        <v>210</v>
-      </c>
-      <c r="G18" s="15" t="s">
+      <c r="F18" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="G18" s="14" t="s">
+        <v>210</v>
+      </c>
+      <c r="H18" s="15" t="s">
         <v>285</v>
       </c>
-      <c r="H18" s="15" t="s">
+      <c r="I18" s="15" t="s">
         <v>286</v>
       </c>
-      <c r="I18" s="16" t="s">
+      <c r="J18" s="16" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="173.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="87"/>
+    <row r="19" spans="1:10" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="99"/>
       <c r="B19" s="14">
         <v>40824</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="68">
+        <v>40805.290972222225</v>
+      </c>
+      <c r="D19" s="14" t="s">
         <v>283</v>
       </c>
-      <c r="D19" s="14" t="s">
-        <v>210</v>
-      </c>
-      <c r="E19" s="14"/>
+      <c r="E19" s="14" t="s">
+        <v>210</v>
+      </c>
       <c r="F19" s="14"/>
-      <c r="G19" s="15" t="s">
+      <c r="G19" s="14"/>
+      <c r="H19" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="H19" s="15" t="s">
+      <c r="I19" s="15" t="s">
         <v>278</v>
       </c>
-      <c r="I19" s="17" t="s">
+      <c r="J19" s="17" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="31">
         <v>2012</v>
       </c>
       <c r="B20" s="26" t="s">
         <v>289</v>
       </c>
-      <c r="C20" s="26" t="s">
+      <c r="C20" s="72">
+        <v>41132.474305555559</v>
+      </c>
+      <c r="D20" s="26" t="s">
         <v>283</v>
       </c>
-      <c r="D20" s="26" t="s">
-        <v>210</v>
-      </c>
-      <c r="E20" s="26"/>
+      <c r="E20" s="26" t="s">
+        <v>210</v>
+      </c>
       <c r="F20" s="26"/>
-      <c r="G20" s="26" t="s">
+      <c r="G20" s="26"/>
+      <c r="H20" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="H20" s="26" t="s">
+      <c r="I20" s="26" t="s">
         <v>288</v>
       </c>
-      <c r="I20" s="27" t="s">
+      <c r="J20" s="27" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="86">
+    <row r="21" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="98">
         <v>2013</v>
       </c>
       <c r="B21" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="67">
+        <v>41291.492361111108</v>
+      </c>
+      <c r="D21" s="12" t="s">
         <v>250</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="E21" s="12" t="s">
         <v>211</v>
       </c>
-      <c r="E21" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12" t="s">
+      <c r="F21" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="H21" s="12"/>
-      <c r="I21" s="13" t="s">
+      <c r="I21" s="12"/>
+      <c r="J21" s="13" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="72" x14ac:dyDescent="0.3">
-      <c r="A22" s="87"/>
+    <row r="22" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="99"/>
       <c r="B22" s="14">
         <v>41310</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="C22" s="68">
+        <v>41306.220138888886</v>
+      </c>
+      <c r="D22" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="E22" s="14" t="s">
         <v>269</v>
       </c>
-      <c r="E22" s="14"/>
       <c r="F22" s="14"/>
-      <c r="G22" s="15" t="s">
+      <c r="G22" s="14"/>
+      <c r="H22" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="H22" s="15"/>
-      <c r="I22" s="16"/>
-    </row>
-    <row r="23" spans="1:9" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="87"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="16"/>
+    </row>
+    <row r="23" spans="1:10" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="99"/>
       <c r="B23" s="14">
         <v>41326</v>
       </c>
-      <c r="C23" s="14" t="s">
+      <c r="C23" s="68">
+        <v>41320.779861111114</v>
+      </c>
+      <c r="D23" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="D23" s="14" t="s">
+      <c r="E23" s="14" t="s">
         <v>211</v>
       </c>
-      <c r="E23" s="14" t="s">
-        <v>210</v>
-      </c>
-      <c r="F23" s="14"/>
-      <c r="G23" s="15" t="s">
+      <c r="F23" s="14" t="s">
+        <v>210</v>
+      </c>
+      <c r="G23" s="14"/>
+      <c r="H23" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="H23" s="15" t="s">
+      <c r="I23" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="I23" s="16" t="s">
+      <c r="J23" s="16" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="202.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="88"/>
+    <row r="24" spans="1:10" ht="202.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="100"/>
       <c r="B24" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="C24" s="71">
+        <v>41358.106944444444</v>
+      </c>
+      <c r="D24" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="D24" s="19" t="s">
+      <c r="E24" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="E24" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19" t="s">
+      <c r="F24" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="G24" s="19"/>
+      <c r="H24" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H24" s="19" t="s">
+      <c r="I24" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="I24" s="17" t="s">
+      <c r="J24" s="17" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A25" s="72">
+    <row r="25" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="84">
         <v>2014</v>
       </c>
       <c r="B25" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="C25" s="12" t="s">
+      <c r="C25" s="67">
+        <v>41723.123611111114</v>
+      </c>
+      <c r="D25" s="12" t="s">
         <v>283</v>
       </c>
-      <c r="D25" s="12" t="s">
+      <c r="E25" s="12" t="s">
         <v>211</v>
       </c>
-      <c r="E25" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="F25" s="12"/>
+      <c r="F25" s="12" t="s">
+        <v>210</v>
+      </c>
       <c r="G25" s="12"/>
       <c r="H25" s="12"/>
-      <c r="I25" s="13" t="s">
+      <c r="I25" s="12"/>
+      <c r="J25" s="13" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="73"/>
+    <row r="26" spans="1:10" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="85"/>
       <c r="B26" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="C26" s="19" t="s">
+      <c r="C26" s="69">
+        <v>41942.446527777778</v>
+      </c>
+      <c r="D26" s="19" t="s">
         <v>283</v>
       </c>
-      <c r="D26" s="19" t="s">
+      <c r="E26" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="E26" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="F26" s="19"/>
+      <c r="F26" s="19" t="s">
+        <v>210</v>
+      </c>
       <c r="G26" s="19"/>
       <c r="H26" s="19"/>
-      <c r="I26" s="17" t="s">
+      <c r="I26" s="19"/>
+      <c r="J26" s="17" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="159" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="86">
+    <row r="27" spans="1:10" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="98">
         <v>2016</v>
       </c>
       <c r="B27" s="11">
         <v>42416</v>
       </c>
-      <c r="C27" s="11" t="s">
+      <c r="C27" s="67">
+        <v>42413.843055555553</v>
+      </c>
+      <c r="D27" s="11" t="s">
         <v>283</v>
       </c>
-      <c r="D27" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="E27" s="11"/>
+      <c r="E27" s="11" t="s">
+        <v>210</v>
+      </c>
       <c r="F27" s="11"/>
-      <c r="G27" s="12" t="s">
+      <c r="G27" s="11"/>
+      <c r="H27" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="H27" s="12"/>
-      <c r="I27" s="13" t="s">
+      <c r="I27" s="12"/>
+      <c r="J27" s="13" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="88"/>
+    <row r="28" spans="1:10" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="100"/>
       <c r="B28" s="43" t="s">
         <v>80</v>
       </c>
-      <c r="C28" s="43" t="s">
+      <c r="C28" s="75">
+        <v>42569.087500000001</v>
+      </c>
+      <c r="D28" s="43" t="s">
         <v>283</v>
       </c>
-      <c r="D28" s="43" t="s">
+      <c r="E28" s="43" t="s">
         <v>241</v>
       </c>
-      <c r="E28" s="43"/>
       <c r="F28" s="43"/>
-      <c r="G28" s="43" t="s">
+      <c r="G28" s="43"/>
+      <c r="H28" s="43" t="s">
         <v>79</v>
       </c>
-      <c r="H28" s="43"/>
-      <c r="I28" s="20"/>
-    </row>
-    <row r="29" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A29" s="72">
+      <c r="I28" s="43"/>
+      <c r="J28" s="20"/>
+    </row>
+    <row r="29" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="A29" s="84">
         <v>2017</v>
       </c>
       <c r="B29" s="11">
         <v>42789</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="67">
+        <v>42788.229861111111</v>
+      </c>
+      <c r="D29" s="11" t="s">
         <v>283</v>
       </c>
-      <c r="D29" s="11" t="s">
+      <c r="E29" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="E29" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="F29" s="11"/>
-      <c r="G29" s="12" t="s">
+      <c r="F29" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="G29" s="11"/>
+      <c r="H29" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="H29" s="12" t="s">
+      <c r="I29" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="I29" s="13" t="s">
+      <c r="J29" s="13" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="206.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="73"/>
+    <row r="30" spans="1:10" ht="206.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="85"/>
       <c r="B30" s="18">
         <v>43089</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="69">
+        <v>43087.26666666667</v>
+      </c>
+      <c r="D30" s="18" t="s">
         <v>283</v>
       </c>
-      <c r="D30" s="18" t="s">
+      <c r="E30" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="E30" s="18" t="s">
-        <v>210</v>
-      </c>
-      <c r="F30" s="18"/>
-      <c r="G30" s="19" t="s">
+      <c r="F30" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="G30" s="18"/>
+      <c r="H30" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="H30" s="19" t="s">
+      <c r="I30" s="19" t="s">
         <v>169</v>
       </c>
-      <c r="I30" s="17" t="s">
+      <c r="J30" s="17" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A31" s="87">
+    <row r="31" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="99">
         <v>2018</v>
       </c>
       <c r="B31" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="C31" s="22" t="s">
+      <c r="C31" s="70">
+        <v>43174.863194444442</v>
+      </c>
+      <c r="D31" s="22" t="s">
         <v>283</v>
       </c>
-      <c r="D31" s="22" t="s">
-        <v>210</v>
-      </c>
-      <c r="E31" s="22"/>
+      <c r="E31" s="22" t="s">
+        <v>210</v>
+      </c>
       <c r="F31" s="22"/>
-      <c r="G31" s="22" t="s">
+      <c r="G31" s="22"/>
+      <c r="H31" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="H31" s="22" t="s">
+      <c r="I31" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="I31" s="23" t="s">
+      <c r="J31" s="23" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A32" s="87"/>
+    <row r="32" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A32" s="99"/>
       <c r="B32" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="C32" s="15" t="s">
+      <c r="C32" s="68">
+        <v>43433.469444444447</v>
+      </c>
+      <c r="D32" s="15" t="s">
         <v>283</v>
       </c>
-      <c r="D32" s="15" t="s">
-        <v>210</v>
-      </c>
-      <c r="E32" s="15"/>
+      <c r="E32" s="15" t="s">
+        <v>210</v>
+      </c>
       <c r="F32" s="15"/>
-      <c r="G32" s="15" t="s">
+      <c r="G32" s="15"/>
+      <c r="H32" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="H32" s="15"/>
-      <c r="I32" s="16"/>
-    </row>
-    <row r="33" spans="1:9" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="88"/>
+      <c r="I32" s="15"/>
+      <c r="J32" s="16"/>
+    </row>
+    <row r="33" spans="1:10" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="100"/>
       <c r="B33" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="C33" s="19" t="s">
+      <c r="C33" s="69">
+        <v>43450.80972222222</v>
+      </c>
+      <c r="D33" s="19" t="s">
         <v>283</v>
       </c>
-      <c r="D33" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="E33" s="19"/>
+      <c r="E33" s="19" t="s">
+        <v>210</v>
+      </c>
       <c r="F33" s="19"/>
-      <c r="G33" s="19" t="s">
+      <c r="G33" s="19"/>
+      <c r="H33" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="H33" s="19" t="s">
+      <c r="I33" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="I33" s="17" t="s">
+      <c r="J33" s="17" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="86">
+    <row r="34" spans="1:10" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="98">
         <v>2021</v>
       </c>
       <c r="B34" s="11">
         <v>44348</v>
       </c>
-      <c r="C34" s="11" t="s">
+      <c r="C34" s="67">
+        <v>44346.974999999999</v>
+      </c>
+      <c r="D34" s="11" t="s">
         <v>241</v>
       </c>
-      <c r="D34" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="E34" s="11"/>
+      <c r="E34" s="11" t="s">
+        <v>210</v>
+      </c>
       <c r="F34" s="11"/>
-      <c r="G34" s="12" t="s">
+      <c r="G34" s="11"/>
+      <c r="H34" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="H34" s="12"/>
-      <c r="I34" s="13" t="s">
+      <c r="I34" s="12"/>
+      <c r="J34" s="13" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A35" s="88"/>
+    <row r="35" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="100"/>
       <c r="B35" s="18">
         <v>44542</v>
       </c>
-      <c r="C35" s="18" t="s">
+      <c r="C35" s="69">
+        <v>44535.438888888886</v>
+      </c>
+      <c r="D35" s="18" t="s">
         <v>241</v>
       </c>
-      <c r="D35" s="18" t="s">
+      <c r="E35" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="E35" s="18" t="s">
-        <v>210</v>
-      </c>
-      <c r="F35" s="18"/>
-      <c r="G35" s="19" t="s">
+      <c r="F35" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="G35" s="18"/>
+      <c r="H35" s="19" t="s">
         <v>170</v>
       </c>
-      <c r="H35" s="19"/>
-      <c r="I35" s="17" t="s">
+      <c r="I35" s="19"/>
+      <c r="J35" s="17" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="97">
+    <row r="36" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A36" s="119">
         <v>2022</v>
       </c>
       <c r="B36" s="11">
         <v>44646</v>
       </c>
-      <c r="C36" s="11" t="s">
+      <c r="C36" s="67">
+        <v>44633.436805555553</v>
+      </c>
+      <c r="D36" s="11" t="s">
         <v>241</v>
       </c>
-      <c r="D36" s="11" t="s">
+      <c r="E36" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="E36" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="F36" s="11"/>
-      <c r="G36" s="12" t="s">
+      <c r="F36" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="G36" s="11"/>
+      <c r="H36" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="H36" s="12" t="s">
+      <c r="I36" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="I36" s="13" t="s">
+      <c r="J36" s="13" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="87" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="98"/>
+    <row r="37" spans="1:10" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="120"/>
       <c r="B37" s="18">
         <v>44873</v>
       </c>
-      <c r="C37" s="18" t="s">
+      <c r="C37" s="69">
+        <v>44875.234027777777</v>
+      </c>
+      <c r="D37" s="18" t="s">
         <v>241</v>
       </c>
-      <c r="D37" s="18" t="s">
+      <c r="E37" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="E37" s="18" t="s">
-        <v>210</v>
-      </c>
-      <c r="F37" s="18"/>
-      <c r="G37" s="19" t="s">
+      <c r="F37" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="G37" s="18"/>
+      <c r="H37" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="H37" s="19"/>
-      <c r="I37" s="17" t="s">
+      <c r="I37" s="19"/>
+      <c r="J37" s="17" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" ht="58.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="51">
         <v>2023</v>
       </c>
       <c r="B38" s="35">
         <v>44950</v>
       </c>
-      <c r="C38" s="35" t="s">
+      <c r="C38" s="72">
+        <v>44939.754166666666</v>
+      </c>
+      <c r="D38" s="35" t="s">
         <v>241</v>
       </c>
-      <c r="D38" s="35" t="s">
-        <v>210</v>
-      </c>
-      <c r="E38" s="35"/>
+      <c r="E38" s="35" t="s">
+        <v>210</v>
+      </c>
       <c r="F38" s="35"/>
-      <c r="G38" s="26" t="s">
+      <c r="G38" s="35"/>
+      <c r="H38" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="H38" s="26" t="s">
+      <c r="I38" s="26" t="s">
         <v>292</v>
       </c>
-      <c r="I38" s="27" t="s">
+      <c r="J38" s="27" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" ht="63" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="10">
         <v>2025</v>
       </c>
       <c r="B39" s="35">
         <v>45826</v>
       </c>
-      <c r="C39" s="35" t="s">
+      <c r="C39" s="72">
+        <v>45821.534722222219</v>
+      </c>
+      <c r="D39" s="35" t="s">
         <v>241</v>
       </c>
-      <c r="D39" s="35" t="s">
+      <c r="E39" s="35" t="s">
         <v>211</v>
       </c>
-      <c r="E39" s="35" t="s">
-        <v>210</v>
-      </c>
-      <c r="F39" s="35"/>
-      <c r="G39" s="26" t="s">
+      <c r="F39" s="35" t="s">
+        <v>210</v>
+      </c>
+      <c r="G39" s="35"/>
+      <c r="H39" s="26" t="s">
         <v>101</v>
       </c>
-      <c r="H39" s="26"/>
-      <c r="I39" s="27" t="s">
+      <c r="I39" s="26"/>
+      <c r="J39" s="27" t="s">
         <v>102</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I39" xr:uid="{B1F67599-3BD8-474A-B2DB-71494680CF1C}"/>
+  <autoFilter ref="A4:J39" xr:uid="{B1F67599-3BD8-474A-B2DB-71494680CF1C}"/>
   <mergeCells count="20">
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
     <mergeCell ref="B14:B15"/>
-    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="G14:G15"/>
     <mergeCell ref="A36:A37"/>
     <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A1:I3"/>
+    <mergeCell ref="A1:J3"/>
     <mergeCell ref="A5:A8"/>
     <mergeCell ref="A11:A13"/>
     <mergeCell ref="A31:A33"/>
@@ -4451,13 +4735,16 @@
     <mergeCell ref="A25:A26"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="A29:A30"/>
-    <mergeCell ref="G14:G15"/>
     <mergeCell ref="H14:H15"/>
     <mergeCell ref="I14:I15"/>
-    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="F14:F15"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;R_x000D_&amp;1#&amp;"Aptos"&amp;22&amp;KFF8939 RESTRICTED</oddFooter>
   </headerFooter>
@@ -4466,823 +4753,927 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC3F29DD-DB65-4C35-AB17-C9DBDC359F34}">
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="18.109375" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" customWidth="1"/>
-    <col min="4" max="6" width="18.109375" customWidth="1"/>
-    <col min="7" max="7" width="53.5546875" customWidth="1"/>
-    <col min="8" max="8" width="44" customWidth="1"/>
-    <col min="9" max="9" width="37.109375" customWidth="1"/>
+    <col min="1" max="1" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="56.44140625" style="76" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="65.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="62" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="44.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="103" t="s">
+    <row r="1" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="121" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="104"/>
-      <c r="C1" s="104"/>
-      <c r="D1" s="104"/>
-      <c r="E1" s="104"/>
-      <c r="F1" s="104"/>
-      <c r="G1" s="104"/>
-      <c r="H1" s="104"/>
-      <c r="I1" s="105"/>
-    </row>
-    <row r="2" spans="1:9" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="106"/>
-      <c r="B2" s="107"/>
-      <c r="C2" s="107"/>
-      <c r="D2" s="107"/>
-      <c r="E2" s="107"/>
-      <c r="F2" s="107"/>
-      <c r="G2" s="107"/>
-      <c r="H2" s="107"/>
-      <c r="I2" s="108"/>
-    </row>
-    <row r="3" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="109"/>
-      <c r="B3" s="110"/>
-      <c r="C3" s="110"/>
-      <c r="D3" s="110"/>
-      <c r="E3" s="110"/>
-      <c r="F3" s="110"/>
-      <c r="G3" s="110"/>
-      <c r="H3" s="110"/>
-      <c r="I3" s="111"/>
-    </row>
-    <row r="4" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="122"/>
+      <c r="C1" s="122"/>
+      <c r="D1" s="122"/>
+      <c r="E1" s="122"/>
+      <c r="F1" s="122"/>
+      <c r="G1" s="122"/>
+      <c r="H1" s="122"/>
+      <c r="I1" s="122"/>
+      <c r="J1" s="123"/>
+    </row>
+    <row r="2" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="124"/>
+      <c r="B2" s="125"/>
+      <c r="C2" s="125"/>
+      <c r="D2" s="125"/>
+      <c r="E2" s="125"/>
+      <c r="F2" s="125"/>
+      <c r="G2" s="125"/>
+      <c r="H2" s="125"/>
+      <c r="I2" s="125"/>
+      <c r="J2" s="126"/>
+    </row>
+    <row r="3" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="127"/>
+      <c r="B3" s="128"/>
+      <c r="C3" s="128"/>
+      <c r="D3" s="128"/>
+      <c r="E3" s="128"/>
+      <c r="F3" s="128"/>
+      <c r="G3" s="128"/>
+      <c r="H3" s="128"/>
+      <c r="I3" s="128"/>
+      <c r="J3" s="129"/>
+    </row>
+    <row r="4" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="78" t="s">
+        <v>306</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="I4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="J4" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="114" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="114" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7">
         <v>2003</v>
       </c>
       <c r="B5" s="59">
         <v>37841</v>
       </c>
-      <c r="C5" s="59" t="s">
+      <c r="C5" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D5" s="59" t="s">
         <v>283</v>
       </c>
-      <c r="D5" s="59" t="s">
+      <c r="E5" s="59" t="s">
         <v>211</v>
       </c>
-      <c r="E5" s="59" t="s">
-        <v>210</v>
-      </c>
-      <c r="F5" s="59"/>
-      <c r="G5" s="26" t="s">
+      <c r="F5" s="59" t="s">
+        <v>210</v>
+      </c>
+      <c r="G5" s="59"/>
+      <c r="H5" s="26" t="s">
         <v>171</v>
       </c>
-      <c r="H5" s="60" t="s">
+      <c r="I5" s="60" t="s">
         <v>172</v>
       </c>
-      <c r="I5" s="61"/>
-    </row>
-    <row r="6" spans="1:9" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="84">
+      <c r="J5" s="61"/>
+    </row>
+    <row r="6" spans="1:10" ht="159" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="96">
         <v>2004</v>
       </c>
       <c r="B6" s="38">
         <v>38069</v>
       </c>
-      <c r="C6" s="44" t="s">
+      <c r="C6" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D6" s="44" t="s">
         <v>279</v>
       </c>
-      <c r="D6" s="38" t="s">
+      <c r="E6" s="38" t="s">
         <v>211</v>
       </c>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38" t="s">
-        <v>210</v>
-      </c>
-      <c r="G6" s="12" t="s">
+      <c r="F6" s="38"/>
+      <c r="G6" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="H6" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="H6" s="36"/>
-      <c r="I6" s="58"/>
-    </row>
-    <row r="7" spans="1:9" ht="173.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="85"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="58"/>
+    </row>
+    <row r="7" spans="1:10" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="97"/>
       <c r="B7" s="56">
         <v>38287</v>
       </c>
-      <c r="C7" s="56" t="s">
+      <c r="C7" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D7" s="56" t="s">
         <v>283</v>
       </c>
-      <c r="D7" s="56" t="s">
+      <c r="E7" s="56" t="s">
         <v>211</v>
       </c>
-      <c r="E7" s="56"/>
       <c r="F7" s="56"/>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="56"/>
+      <c r="H7" s="19" t="s">
         <v>175</v>
       </c>
-      <c r="H7" s="57" t="s">
+      <c r="I7" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="I7" s="17" t="s">
+      <c r="J7" s="17" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="144" x14ac:dyDescent="0.3">
-      <c r="A8" s="91">
+    <row r="8" spans="1:10" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="103">
         <v>2005</v>
       </c>
       <c r="B8" s="38">
         <v>38481</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="C8" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D8" s="44" t="s">
         <v>279</v>
       </c>
-      <c r="D8" s="38" t="s">
+      <c r="E8" s="38" t="s">
         <v>211</v>
       </c>
-      <c r="E8" s="38" t="s">
-        <v>210</v>
-      </c>
-      <c r="F8" s="38"/>
-      <c r="G8" s="12" t="s">
+      <c r="F8" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="G8" s="38"/>
+      <c r="H8" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="H8" s="36"/>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="36"/>
+      <c r="J8" s="13" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="92"/>
+    <row r="9" spans="1:10" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="104"/>
       <c r="B9" s="39" t="s">
         <v>294</v>
       </c>
-      <c r="C9" s="39" t="s">
+      <c r="C9" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D9" s="39" t="s">
         <v>283</v>
       </c>
-      <c r="D9" s="39" t="s">
-        <v>210</v>
-      </c>
       <c r="E9" s="39" t="s">
         <v>210</v>
       </c>
-      <c r="F9" s="39"/>
-      <c r="G9" s="15" t="s">
+      <c r="F9" s="39" t="s">
+        <v>210</v>
+      </c>
+      <c r="G9" s="39"/>
+      <c r="H9" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="H9" s="40" t="s">
+      <c r="I9" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="I9" s="16" t="s">
+      <c r="J9" s="16" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="93"/>
+    <row r="10" spans="1:10" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="105"/>
       <c r="B10" s="41" t="s">
         <v>295</v>
       </c>
-      <c r="C10" s="41" t="s">
+      <c r="C10" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D10" s="41" t="s">
         <v>283</v>
       </c>
-      <c r="D10" s="41" t="s">
-        <v>210</v>
-      </c>
       <c r="E10" s="41" t="s">
         <v>210</v>
       </c>
-      <c r="F10" s="41"/>
-      <c r="G10" s="19" t="s">
+      <c r="F10" s="41" t="s">
+        <v>210</v>
+      </c>
+      <c r="G10" s="41"/>
+      <c r="H10" s="19" t="s">
         <v>180</v>
       </c>
-      <c r="H10" s="50" t="s">
+      <c r="I10" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="I10" s="17" t="s">
+      <c r="J10" s="17" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="173.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="37">
         <v>2007</v>
       </c>
       <c r="B11" s="62">
         <v>39168</v>
       </c>
-      <c r="C11" s="62" t="s">
+      <c r="C11" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D11" s="62" t="s">
         <v>283</v>
       </c>
-      <c r="D11" s="62" t="s">
-        <v>210</v>
-      </c>
       <c r="E11" s="62" t="s">
         <v>210</v>
       </c>
-      <c r="F11" s="62"/>
-      <c r="G11" s="26" t="s">
+      <c r="F11" s="62" t="s">
+        <v>210</v>
+      </c>
+      <c r="G11" s="62"/>
+      <c r="H11" s="26" t="s">
         <v>296</v>
       </c>
-      <c r="H11" s="26" t="s">
+      <c r="I11" s="26" t="s">
         <v>267</v>
       </c>
-      <c r="I11" s="27" t="s">
+      <c r="J11" s="27" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="72" x14ac:dyDescent="0.3">
-      <c r="A12" s="91">
+    <row r="12" spans="1:10" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="103">
         <v>2008</v>
       </c>
       <c r="B12" s="44">
         <v>39548</v>
       </c>
-      <c r="C12" s="44" t="s">
+      <c r="C12" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D12" s="44" t="s">
         <v>283</v>
       </c>
-      <c r="D12" s="44" t="s">
-        <v>210</v>
-      </c>
-      <c r="E12" s="44"/>
+      <c r="E12" s="44" t="s">
+        <v>210</v>
+      </c>
       <c r="F12" s="44"/>
-      <c r="G12" s="12" t="s">
+      <c r="G12" s="44"/>
+      <c r="H12" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H12" s="12" t="s">
+      <c r="I12" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="I12" s="13" t="s">
+      <c r="J12" s="13" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="92"/>
+    <row r="13" spans="1:10" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="104"/>
       <c r="B13" s="39">
         <v>39728</v>
       </c>
-      <c r="C13" s="41" t="s">
+      <c r="C13" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D13" s="41" t="s">
         <v>279</v>
       </c>
-      <c r="D13" s="39"/>
       <c r="E13" s="39"/>
       <c r="F13" s="39"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15" t="s">
+      <c r="G13" s="39"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15" t="s">
         <v>303</v>
       </c>
-      <c r="I13" s="16"/>
-    </row>
-    <row r="14" spans="1:9" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="93"/>
+      <c r="J13" s="16"/>
+    </row>
+    <row r="14" spans="1:10" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="105"/>
       <c r="B14" s="41">
         <v>39797</v>
       </c>
-      <c r="C14" s="41" t="s">
+      <c r="C14" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D14" s="41" t="s">
         <v>279</v>
       </c>
-      <c r="D14" s="41" t="s">
-        <v>210</v>
-      </c>
-      <c r="E14" s="41"/>
+      <c r="E14" s="41" t="s">
+        <v>210</v>
+      </c>
       <c r="F14" s="41"/>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="41"/>
+      <c r="H14" s="19" t="s">
         <v>184</v>
       </c>
-      <c r="H14" s="19" t="s">
+      <c r="I14" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="I14" s="17" t="s">
+      <c r="J14" s="17" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="103.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="84">
+    <row r="15" spans="1:10" ht="103.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="96">
         <v>2009</v>
       </c>
       <c r="B15" s="11">
         <v>39909</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D15" s="11" t="s">
         <v>279</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="E15" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="E15" s="11"/>
       <c r="F15" s="11"/>
-      <c r="G15" s="12" t="s">
+      <c r="G15" s="11"/>
+      <c r="H15" s="12" t="s">
         <v>186</v>
       </c>
-      <c r="H15" s="12"/>
-      <c r="I15" s="58"/>
-    </row>
-    <row r="16" spans="1:9" ht="159" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="85"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="58"/>
+    </row>
+    <row r="16" spans="1:10" ht="159" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="97"/>
       <c r="B16" s="63" t="s">
         <v>298</v>
       </c>
-      <c r="C16" s="63" t="s">
+      <c r="C16" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D16" s="63" t="s">
         <v>283</v>
       </c>
-      <c r="D16" s="63" t="s">
-        <v>210</v>
-      </c>
-      <c r="E16" s="63"/>
+      <c r="E16" s="63" t="s">
+        <v>210</v>
+      </c>
       <c r="F16" s="63"/>
-      <c r="G16" s="64" t="s">
+      <c r="G16" s="63"/>
+      <c r="H16" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="H16" s="64" t="s">
+      <c r="I16" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="I16" s="65" t="s">
+      <c r="J16" s="65" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="231" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" ht="202.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
         <v>2010</v>
       </c>
       <c r="B17" s="35">
         <v>40513</v>
       </c>
-      <c r="C17" s="35" t="s">
+      <c r="C17" s="67" t="s">
+        <v>307</v>
+      </c>
+      <c r="D17" s="35" t="s">
         <v>283</v>
       </c>
-      <c r="D17" s="35" t="s">
-        <v>210</v>
-      </c>
       <c r="E17" s="35" t="s">
         <v>210</v>
       </c>
       <c r="F17" s="35" t="s">
         <v>210</v>
       </c>
-      <c r="G17" s="26" t="s">
+      <c r="G17" s="35" t="s">
+        <v>210</v>
+      </c>
+      <c r="H17" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="H17" s="26" t="s">
+      <c r="I17" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="I17" s="27" t="s">
+      <c r="J17" s="27" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="28">
         <v>2012</v>
       </c>
       <c r="B18" s="54" t="s">
         <v>299</v>
       </c>
-      <c r="C18" s="54" t="s">
+      <c r="C18" s="77">
+        <v>41000.491666666669</v>
+      </c>
+      <c r="D18" s="54" t="s">
         <v>283</v>
       </c>
-      <c r="D18" s="54" t="s">
+      <c r="E18" s="54" t="s">
         <v>211</v>
       </c>
-      <c r="E18" s="54" t="s">
-        <v>210</v>
-      </c>
-      <c r="F18" s="54"/>
-      <c r="G18" s="52"/>
-      <c r="H18" s="52" t="s">
+      <c r="F18" s="54" t="s">
+        <v>210</v>
+      </c>
+      <c r="G18" s="54"/>
+      <c r="H18" s="52"/>
+      <c r="I18" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="I18" s="53" t="s">
+      <c r="J18" s="53" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="389.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" ht="331.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="7">
         <v>2013</v>
       </c>
       <c r="B19" s="35">
         <v>41602</v>
       </c>
-      <c r="C19" s="35" t="s">
+      <c r="C19" s="72">
+        <v>41601.502083333333</v>
+      </c>
+      <c r="D19" s="35" t="s">
         <v>283</v>
       </c>
-      <c r="D19" s="35" t="s">
-        <v>210</v>
-      </c>
-      <c r="E19" s="35"/>
+      <c r="E19" s="35" t="s">
+        <v>210</v>
+      </c>
       <c r="F19" s="35"/>
-      <c r="G19" s="55" t="s">
+      <c r="G19" s="35"/>
+      <c r="H19" s="55" t="s">
         <v>190</v>
       </c>
-      <c r="H19" s="26" t="s">
+      <c r="I19" s="26" t="s">
         <v>189</v>
       </c>
-      <c r="I19" s="27" t="s">
+      <c r="J19" s="27" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="29">
         <v>2015</v>
       </c>
       <c r="B20" s="42">
         <v>42045</v>
       </c>
-      <c r="C20" s="42" t="s">
+      <c r="C20" s="75">
+        <v>42044.909722222219</v>
+      </c>
+      <c r="D20" s="42" t="s">
         <v>283</v>
       </c>
-      <c r="D20" s="42" t="s">
-        <v>210</v>
-      </c>
-      <c r="E20" s="42"/>
+      <c r="E20" s="42" t="s">
+        <v>210</v>
+      </c>
       <c r="F20" s="42"/>
-      <c r="G20" s="43" t="s">
+      <c r="G20" s="42"/>
+      <c r="H20" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="H20" s="43" t="s">
+      <c r="I20" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="I20" s="20" t="s">
+      <c r="J20" s="20" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="144" x14ac:dyDescent="0.3">
-      <c r="A21" s="91">
+    <row r="21" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="103">
         <v>2017</v>
       </c>
       <c r="B21" s="11" t="s">
         <v>301</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="67" t="s">
+        <v>241</v>
+      </c>
+      <c r="D21" s="11" t="s">
         <v>283</v>
       </c>
-      <c r="D21" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="E21" s="11"/>
+      <c r="E21" s="11" t="s">
+        <v>210</v>
+      </c>
       <c r="F21" s="11"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="12" t="s">
+      <c r="G21" s="11"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12" t="s">
         <v>192</v>
       </c>
-      <c r="I21" s="13" t="s">
+      <c r="J21" s="13" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="92"/>
+    <row r="22" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A22" s="104"/>
       <c r="B22" s="14" t="s">
         <v>302</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="C22" s="68">
+        <v>43036.112500000003</v>
+      </c>
+      <c r="D22" s="14" t="s">
         <v>283</v>
       </c>
-      <c r="D22" s="14" t="s">
-        <v>210</v>
-      </c>
-      <c r="E22" s="14"/>
+      <c r="E22" s="14" t="s">
+        <v>210</v>
+      </c>
       <c r="F22" s="14"/>
-      <c r="G22" s="15" t="s">
+      <c r="G22" s="14"/>
+      <c r="H22" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="H22" s="15" t="s">
+      <c r="I22" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="I22" s="16" t="s">
+      <c r="J22" s="16" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="93"/>
+    <row r="23" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="105"/>
       <c r="B23" s="18">
         <v>43081</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="69">
+        <v>43079.443749999999</v>
+      </c>
+      <c r="D23" s="18" t="s">
         <v>283</v>
       </c>
-      <c r="D23" s="18" t="s">
+      <c r="E23" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="E23" s="18" t="s">
-        <v>210</v>
-      </c>
-      <c r="F23" s="18"/>
-      <c r="G23" s="19"/>
+      <c r="F23" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="G23" s="18"/>
       <c r="H23" s="19"/>
-      <c r="I23" s="17" t="s">
+      <c r="I23" s="19"/>
+      <c r="J23" s="17" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="84">
+    <row r="24" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="96">
         <v>2018</v>
       </c>
       <c r="B24" s="11">
         <v>43181</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="67">
+        <v>43181.644444444442</v>
+      </c>
+      <c r="D24" s="11" t="s">
         <v>283</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="E24" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="E24" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="F24" s="11"/>
-      <c r="G24" s="12" t="s">
+      <c r="F24" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="G24" s="11"/>
+      <c r="H24" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="H24" s="12"/>
-      <c r="I24" s="13" t="s">
+      <c r="I24" s="12"/>
+      <c r="J24" s="13" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="87" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="85"/>
+    <row r="25" spans="1:10" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="97"/>
       <c r="B25" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="C25" s="18" t="s">
+      <c r="C25" s="69">
+        <v>43314.782638888886</v>
+      </c>
+      <c r="D25" s="18" t="s">
         <v>283</v>
       </c>
-      <c r="D25" s="18" t="s">
+      <c r="E25" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="E25" s="18"/>
       <c r="F25" s="18"/>
-      <c r="G25" s="19" t="s">
+      <c r="G25" s="18"/>
+      <c r="H25" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H25" s="19" t="s">
+      <c r="I25" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="I25" s="17" t="s">
+      <c r="J25" s="17" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="91">
+    <row r="26" spans="1:10" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="103">
         <v>2019</v>
       </c>
       <c r="B26" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="67">
+        <v>43556.920138888891</v>
+      </c>
+      <c r="D26" s="11" t="s">
         <v>283</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="E26" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="E26" s="11"/>
       <c r="F26" s="11"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="12" t="s">
+      <c r="G26" s="11"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="I26" s="13"/>
-    </row>
-    <row r="27" spans="1:9" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="93"/>
+      <c r="J26" s="13"/>
+    </row>
+    <row r="27" spans="1:10" ht="187.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="105"/>
       <c r="B27" s="41" t="s">
         <v>29</v>
       </c>
-      <c r="C27" s="41" t="s">
+      <c r="C27" s="67">
+        <v>43556.920138888891</v>
+      </c>
+      <c r="D27" s="41" t="s">
         <v>283</v>
       </c>
-      <c r="D27" s="41" t="s">
+      <c r="E27" s="41" t="s">
         <v>211</v>
       </c>
-      <c r="E27" s="41" t="s">
-        <v>210</v>
-      </c>
-      <c r="F27" s="41"/>
-      <c r="G27" s="19" t="s">
+      <c r="F27" s="41" t="s">
+        <v>210</v>
+      </c>
+      <c r="G27" s="41"/>
+      <c r="H27" s="19" t="s">
         <v>291</v>
       </c>
-      <c r="H27" s="19" t="s">
+      <c r="I27" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="I27" s="17" t="s">
+      <c r="J27" s="17" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="29">
         <v>2020</v>
       </c>
       <c r="B28" s="42" t="s">
         <v>305</v>
       </c>
-      <c r="C28" s="42" t="s">
+      <c r="C28" s="75" t="s">
+        <v>241</v>
+      </c>
+      <c r="D28" s="42" t="s">
         <v>283</v>
       </c>
-      <c r="D28" s="42" t="s">
-        <v>210</v>
-      </c>
-      <c r="E28" s="42"/>
+      <c r="E28" s="42" t="s">
+        <v>210</v>
+      </c>
       <c r="F28" s="42"/>
-      <c r="G28" s="43" t="s">
+      <c r="G28" s="42"/>
+      <c r="H28" s="43" t="s">
         <v>198</v>
       </c>
-      <c r="H28" s="22" t="s">
+      <c r="I28" s="22" t="s">
         <v>196</v>
       </c>
-      <c r="I28" s="23" t="s">
+      <c r="J28" s="23" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A29" s="91">
+    <row r="29" spans="1:10" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="103">
         <v>2021</v>
       </c>
       <c r="B29" s="11">
         <v>44305</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="67">
+        <v>44305.12777777778</v>
+      </c>
+      <c r="D29" s="11" t="s">
         <v>241</v>
       </c>
-      <c r="D29" s="11" t="s">
+      <c r="E29" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="E29" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="F29" s="11"/>
-      <c r="G29" s="12" t="s">
+      <c r="F29" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="G29" s="11"/>
+      <c r="H29" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="H29" s="12"/>
-      <c r="I29" s="12" t="s">
+      <c r="I29" s="12"/>
+      <c r="J29" s="12" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="93"/>
+    <row r="30" spans="1:10" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="105"/>
       <c r="B30" s="18">
         <v>44470</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="69" t="s">
         <v>241</v>
       </c>
       <c r="D30" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="E30" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="E30" s="18"/>
       <c r="F30" s="18"/>
-      <c r="G30" s="19" t="s">
+      <c r="G30" s="18"/>
+      <c r="H30" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="H30" s="19" t="s">
+      <c r="I30" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="I30" s="17"/>
-    </row>
-    <row r="31" spans="1:9" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="J30" s="17"/>
+    </row>
+    <row r="31" spans="1:10" ht="37.200000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="28">
         <v>2022</v>
       </c>
       <c r="B31" s="11">
         <v>44709</v>
       </c>
-      <c r="C31" s="11" t="s">
+      <c r="C31" s="67">
+        <v>44704.615972222222</v>
+      </c>
+      <c r="D31" s="11" t="s">
         <v>241</v>
       </c>
-      <c r="D31" s="11" t="s">
+      <c r="E31" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="E31" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="F31" s="11"/>
-      <c r="G31" s="12"/>
+      <c r="F31" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="G31" s="11"/>
       <c r="H31" s="12"/>
-      <c r="I31" s="12" t="s">
+      <c r="I31" s="12"/>
+      <c r="J31" s="12" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A32" s="91">
+    <row r="32" spans="1:10" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="103">
         <v>2023</v>
       </c>
       <c r="B32" s="44">
         <v>45135</v>
       </c>
-      <c r="C32" s="44" t="s">
+      <c r="C32" s="80" t="s">
         <v>241</v>
       </c>
       <c r="D32" s="44" t="s">
+        <v>241</v>
+      </c>
+      <c r="E32" s="44" t="s">
         <v>211</v>
       </c>
-      <c r="E32" s="44" t="s">
-        <v>210</v>
-      </c>
-      <c r="F32" s="44"/>
-      <c r="G32" s="12" t="s">
+      <c r="F32" s="44" t="s">
+        <v>210</v>
+      </c>
+      <c r="G32" s="44"/>
+      <c r="H32" s="12" t="s">
         <v>270</v>
       </c>
-      <c r="H32" s="12"/>
-      <c r="I32" s="13" t="s">
+      <c r="I32" s="12"/>
+      <c r="J32" s="13" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" s="93"/>
+    <row r="33" spans="1:10" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="105"/>
       <c r="B33" s="41">
         <v>45197</v>
       </c>
-      <c r="C33" s="41" t="s">
+      <c r="C33" s="79">
+        <v>45194.981944444444</v>
+      </c>
+      <c r="D33" s="41" t="s">
         <v>241</v>
       </c>
-      <c r="D33" s="41" t="s">
+      <c r="E33" s="41" t="s">
         <v>211</v>
       </c>
-      <c r="E33" s="41" t="s">
-        <v>210</v>
-      </c>
-      <c r="F33" s="41"/>
-      <c r="G33" s="19" t="s">
+      <c r="F33" s="41" t="s">
+        <v>210</v>
+      </c>
+      <c r="G33" s="41"/>
+      <c r="H33" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="H33" s="19" t="s">
+      <c r="I33" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="I33" s="17"/>
-    </row>
-    <row r="34" spans="1:9" ht="181.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="91">
+      <c r="J33" s="17"/>
+    </row>
+    <row r="34" spans="1:10" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="103">
         <v>2024</v>
       </c>
       <c r="B34" s="44">
         <v>45491</v>
       </c>
-      <c r="C34" s="44" t="s">
+      <c r="C34" s="80">
+        <v>45487.636111111111</v>
+      </c>
+      <c r="D34" s="44" t="s">
         <v>241</v>
       </c>
-      <c r="D34" s="44" t="s">
+      <c r="E34" s="44" t="s">
         <v>211</v>
       </c>
-      <c r="E34" s="44" t="s">
-        <v>210</v>
-      </c>
-      <c r="F34" s="44"/>
-      <c r="G34" s="12" t="s">
+      <c r="F34" s="44" t="s">
+        <v>210</v>
+      </c>
+      <c r="G34" s="44"/>
+      <c r="H34" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="H34" s="12" t="s">
+      <c r="I34" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="I34" s="13" t="s">
+      <c r="J34" s="13" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" s="93"/>
+    <row r="35" spans="1:10" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="105"/>
       <c r="B35" s="41">
         <v>45587</v>
       </c>
-      <c r="C35" s="41" t="s">
+      <c r="C35" s="79">
+        <v>45583.434027777781</v>
+      </c>
+      <c r="D35" s="41" t="s">
         <v>241</v>
       </c>
-      <c r="D35" s="41" t="s">
+      <c r="E35" s="41" t="s">
         <v>211</v>
       </c>
-      <c r="E35" s="41" t="s">
-        <v>210</v>
-      </c>
-      <c r="F35" s="41"/>
-      <c r="G35" s="19" t="s">
+      <c r="F35" s="41" t="s">
+        <v>210</v>
+      </c>
+      <c r="G35" s="41"/>
+      <c r="H35" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="H35" s="19"/>
-      <c r="I35" s="17"/>
-    </row>
+      <c r="I35" s="19"/>
+      <c r="J35" s="17"/>
+    </row>
+    <row r="36" spans="1:10" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <autoFilter ref="A4:I35" xr:uid="{CC3F29DD-DB65-4C35-AB17-C9DBDC359F34}"/>
+  <autoFilter ref="A4:J35" xr:uid="{CC3F29DD-DB65-4C35-AB17-C9DBDC359F34}"/>
   <mergeCells count="11">
     <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A1:I3"/>
+    <mergeCell ref="A1:J3"/>
     <mergeCell ref="A34:A35"/>
     <mergeCell ref="A21:A23"/>
     <mergeCell ref="A24:A25"/>

</xml_diff>